<commit_message>
Add LC Rev sheet
</commit_message>
<xml_diff>
--- a/DSA_Rev.xlsx
+++ b/DSA_Rev.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="40">
   <si>
     <t xml:space="preserve">S.No</t>
   </si>
@@ -238,6 +238,18 @@
     <t xml:space="preserve">use Hashmap to track each node &amp; retrieve, create new if not found in map.if found use same</t>
   </si>
   <si>
+    <t xml:space="preserve">plus-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if Right Most is 9, then add 1 to prev, and make current zero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spiral_matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Boundaries,then go left to right, top to down, right to left, down to up</t>
+  </si>
+  <si>
     <t xml:space="preserve">flatten-a-multilevel-doubly-linked-list</t>
   </si>
   <si>
@@ -396,7 +408,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -457,8 +469,12 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -672,7 +688,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="36.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="36.57"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.55"/>
@@ -810,7 +826,7 @@
         <f aca="false">D4+1</f>
         <v>45703</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="9" t="n">
         <f aca="false">E4+2</f>
         <v>45705</v>
       </c>
@@ -849,7 +865,7 @@
         <f aca="false">D5+1</f>
         <v>45703</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="9" t="n">
         <f aca="false">E5+2</f>
         <v>45705</v>
       </c>
@@ -888,7 +904,7 @@
         <f aca="false">D6+1</f>
         <v>45703</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="9" t="n">
         <f aca="false">E6+2</f>
         <v>45705</v>
       </c>
@@ -927,7 +943,7 @@
         <f aca="false">D7+1</f>
         <v>45703</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="9" t="n">
         <f aca="false">E7+2</f>
         <v>45705</v>
       </c>
@@ -966,7 +982,7 @@
         <f aca="false">D8+1</f>
         <v>45703</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="9" t="n">
         <f aca="false">E8+2</f>
         <v>45705</v>
       </c>
@@ -1005,7 +1021,7 @@
         <f aca="false">D9+1</f>
         <v>45703</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="9" t="n">
         <f aca="false">E9+2</f>
         <v>45705</v>
       </c>
@@ -1155,21 +1171,45 @@
       <c r="D13" s="12" t="n">
         <v>45704</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="11"/>
+      <c r="E13" s="9" t="n">
+        <f aca="false">D13+1</f>
+        <v>45705</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <f aca="false">E13+2</f>
+        <v>45707</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <f aca="false">F13+3</f>
+        <v>45710</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <f aca="false">G13+7</f>
+        <v>45717</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <f aca="false">H13+14</f>
+        <v>45731</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <f aca="false">I13+20</f>
+        <v>45751</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <f aca="false">ROW()-1</f>
         <v>13</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="16"/>
+      <c r="B14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>45705</v>
+      </c>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -1182,9 +1222,15 @@
         <f aca="false">ROW()-1</f>
         <v>14</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>45705</v>
+      </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -1199,7 +1245,7 @@
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="16"/>
+      <c r="D16" s="17"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
@@ -1214,7 +1260,7 @@
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="16"/>
+      <c r="D17" s="17"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -1229,7 +1275,7 @@
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
-      <c r="D18" s="16"/>
+      <c r="D18" s="17"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
@@ -1244,7 +1290,7 @@
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
-      <c r="D19" s="16"/>
+      <c r="D19" s="17"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -1259,7 +1305,7 @@
       </c>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
-      <c r="D20" s="16"/>
+      <c r="D20" s="17"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
@@ -1274,7 +1320,7 @@
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
-      <c r="D21" s="16"/>
+      <c r="D21" s="17"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
@@ -1289,7 +1335,7 @@
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="16"/>
+      <c r="D22" s="17"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
@@ -1304,7 +1350,7 @@
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
-      <c r="D23" s="16"/>
+      <c r="D23" s="17"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
@@ -1319,7 +1365,7 @@
       </c>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
-      <c r="D24" s="16"/>
+      <c r="D24" s="17"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
@@ -1334,7 +1380,7 @@
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
-      <c r="D25" s="16"/>
+      <c r="D25" s="17"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
@@ -1349,7 +1395,7 @@
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
-      <c r="D26" s="16"/>
+      <c r="D26" s="17"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
@@ -1364,7 +1410,7 @@
       </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
-      <c r="D27" s="16"/>
+      <c r="D27" s="17"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
@@ -1379,7 +1425,7 @@
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
-      <c r="D28" s="16"/>
+      <c r="D28" s="17"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
@@ -1394,7 +1440,7 @@
       </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
-      <c r="D29" s="16"/>
+      <c r="D29" s="17"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
@@ -1409,7 +1455,7 @@
       </c>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
-      <c r="D30" s="16"/>
+      <c r="D30" s="17"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
@@ -1424,7 +1470,7 @@
       </c>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
-      <c r="D31" s="16"/>
+      <c r="D31" s="17"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
@@ -1439,7 +1485,7 @@
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
-      <c r="D32" s="16"/>
+      <c r="D32" s="17"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
@@ -1454,7 +1500,7 @@
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
-      <c r="D33" s="16"/>
+      <c r="D33" s="17"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -1469,7 +1515,7 @@
       </c>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
-      <c r="D34" s="16"/>
+      <c r="D34" s="17"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -1484,7 +1530,7 @@
       </c>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
-      <c r="D35" s="16"/>
+      <c r="D35" s="17"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
@@ -1499,7 +1545,7 @@
       </c>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
-      <c r="D36" s="16"/>
+      <c r="D36" s="17"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
       <c r="G36" s="10"/>
@@ -1514,7 +1560,7 @@
       </c>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
-      <c r="D37" s="16"/>
+      <c r="D37" s="17"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
       <c r="G37" s="10"/>
@@ -1523,10 +1569,10 @@
       <c r="J37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
-      <c r="D38" s="16"/>
+      <c r="D38" s="17"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
       <c r="G38" s="10"/>
@@ -1535,10 +1581,10 @@
       <c r="J38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
+      <c r="A39" s="18"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
-      <c r="D39" s="16"/>
+      <c r="D39" s="17"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
@@ -1547,10 +1593,10 @@
       <c r="J39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
+      <c r="A40" s="18"/>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
-      <c r="D40" s="16"/>
+      <c r="D40" s="17"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
@@ -1559,10 +1605,10 @@
       <c r="J40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
+      <c r="A41" s="18"/>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
-      <c r="D41" s="16"/>
+      <c r="D41" s="17"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
       <c r="G41" s="10"/>
@@ -1571,10 +1617,10 @@
       <c r="J41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
+      <c r="A42" s="18"/>
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
-      <c r="D42" s="16"/>
+      <c r="D42" s="17"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
@@ -1583,10 +1629,10 @@
       <c r="J42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
-      <c r="D43" s="16"/>
+      <c r="D43" s="17"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
@@ -1595,10 +1641,10 @@
       <c r="J43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
-      <c r="D44" s="16"/>
+      <c r="D44" s="17"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
@@ -1620,6 +1666,8 @@
     <hyperlink ref="B11" r:id="rId10" display="palindrome-linked-list"/>
     <hyperlink ref="B12" r:id="rId11" display="Design-doubly linkedlist"/>
     <hyperlink ref="B13" r:id="rId12" display="copy-list-with-random-pointer"/>
+    <hyperlink ref="B14" r:id="rId13" display="plus-one"/>
+    <hyperlink ref="B15" r:id="rId14" display="spiral_matrix"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1639,7 +1687,7 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.97"/>
@@ -1683,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D2" s="10" t="n">
@@ -1717,7 +1765,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D3" s="10" t="n">
@@ -1746,9 +1794,9 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -1757,9 +1805,9 @@
       <c r="I4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -1768,9 +1816,9 @@
       <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -1779,9 +1827,9 @@
       <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -1790,9 +1838,9 @@
       <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -1801,9 +1849,9 @@
       <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -1812,9 +1860,9 @@
       <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -1823,9 +1871,9 @@
       <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -1834,9 +1882,9 @@
       <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -1845,9 +1893,9 @@
       <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -1856,9 +1904,9 @@
       <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -1867,9 +1915,9 @@
       <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -1878,9 +1926,9 @@
       <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -1889,9 +1937,9 @@
       <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -1900,9 +1948,9 @@
       <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -1911,9 +1959,9 @@
       <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -1922,9 +1970,9 @@
       <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -1933,9 +1981,9 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -1944,9 +1992,9 @@
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -1955,9 +2003,9 @@
       <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -1966,9 +2014,9 @@
       <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -1977,9 +2025,9 @@
       <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -1988,9 +2036,9 @@
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -1999,9 +2047,9 @@
       <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -2010,9 +2058,9 @@
       <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -2021,9 +2069,9 @@
       <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -2032,9 +2080,9 @@
       <c r="I29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -2043,9 +2091,9 @@
       <c r="I30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -2054,9 +2102,9 @@
       <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -2065,9 +2113,9 @@
       <c r="I32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -2076,9 +2124,9 @@
       <c r="I33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -2087,9 +2135,9 @@
       <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -2098,9 +2146,9 @@
       <c r="I35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -2109,9 +2157,9 @@
       <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -2120,9 +2168,9 @@
       <c r="I37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -2131,9 +2179,9 @@
       <c r="I38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -2142,9 +2190,9 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -2153,9 +2201,9 @@
       <c r="I40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -2164,9 +2212,9 @@
       <c r="I41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -2175,9 +2223,9 @@
       <c r="I42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -2186,9 +2234,9 @@
       <c r="I43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -2215,14 +2263,14 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="19.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="22.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="28.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="18" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="19" width="15.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2260,7 +2308,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D2" s="10" t="n">
@@ -2294,7 +2342,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D3" s="10" t="n">
@@ -2323,9 +2371,9 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -2334,9 +2382,9 @@
       <c r="I4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -2345,9 +2393,9 @@
       <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -2356,9 +2404,9 @@
       <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -2367,9 +2415,9 @@
       <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -2378,9 +2426,9 @@
       <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -2389,9 +2437,9 @@
       <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -2400,9 +2448,9 @@
       <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -2411,9 +2459,9 @@
       <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -2422,9 +2470,9 @@
       <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -2433,9 +2481,9 @@
       <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -2444,9 +2492,9 @@
       <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -2455,9 +2503,9 @@
       <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -2466,9 +2514,9 @@
       <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -2477,9 +2525,9 @@
       <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -2488,9 +2536,9 @@
       <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -2499,9 +2547,9 @@
       <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -2510,9 +2558,9 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -2521,9 +2569,9 @@
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -2532,9 +2580,9 @@
       <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -2543,9 +2591,9 @@
       <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -2554,9 +2602,9 @@
       <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -2565,9 +2613,9 @@
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -2576,9 +2624,9 @@
       <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -2587,9 +2635,9 @@
       <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -2598,9 +2646,9 @@
       <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -2609,9 +2657,9 @@
       <c r="I29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -2620,9 +2668,9 @@
       <c r="I30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -2631,9 +2679,9 @@
       <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -2642,9 +2690,9 @@
       <c r="I32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -2653,9 +2701,9 @@
       <c r="I33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -2664,9 +2712,9 @@
       <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -2675,9 +2723,9 @@
       <c r="I35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -2686,9 +2734,9 @@
       <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -2697,9 +2745,9 @@
       <c r="I37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -2708,9 +2756,9 @@
       <c r="I38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -2719,9 +2767,9 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -2730,9 +2778,9 @@
       <c r="I40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -2741,9 +2789,9 @@
       <c r="I41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -2752,9 +2800,9 @@
       <c r="I42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -2763,9 +2811,9 @@
       <c r="I43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -2792,14 +2840,14 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="19.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="22.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="28.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="18" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="19" width="15.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2837,7 +2885,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D2" s="10" t="n">
@@ -2871,7 +2919,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D3" s="10" t="n">
@@ -2900,9 +2948,9 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -2911,9 +2959,9 @@
       <c r="I4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -2922,9 +2970,9 @@
       <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -2933,9 +2981,9 @@
       <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -2944,9 +2992,9 @@
       <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -2955,9 +3003,9 @@
       <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -2966,9 +3014,9 @@
       <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -2977,9 +3025,9 @@
       <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -2988,9 +3036,9 @@
       <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -2999,9 +3047,9 @@
       <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -3010,9 +3058,9 @@
       <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -3021,9 +3069,9 @@
       <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -3032,9 +3080,9 @@
       <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -3043,9 +3091,9 @@
       <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -3054,9 +3102,9 @@
       <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -3065,9 +3113,9 @@
       <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -3076,9 +3124,9 @@
       <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -3087,9 +3135,9 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -3098,9 +3146,9 @@
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -3109,9 +3157,9 @@
       <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -3120,9 +3168,9 @@
       <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -3131,9 +3179,9 @@
       <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -3142,9 +3190,9 @@
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -3153,9 +3201,9 @@
       <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -3164,9 +3212,9 @@
       <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -3175,9 +3223,9 @@
       <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -3186,9 +3234,9 @@
       <c r="I29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -3197,9 +3245,9 @@
       <c r="I30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -3208,9 +3256,9 @@
       <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -3219,9 +3267,9 @@
       <c r="I32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -3230,9 +3278,9 @@
       <c r="I33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -3241,9 +3289,9 @@
       <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -3252,9 +3300,9 @@
       <c r="I35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -3263,9 +3311,9 @@
       <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -3274,9 +3322,9 @@
       <c r="I37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -3285,9 +3333,9 @@
       <c r="I38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -3296,9 +3344,9 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -3307,9 +3355,9 @@
       <c r="I40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -3318,9 +3366,9 @@
       <c r="I41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -3329,9 +3377,9 @@
       <c r="I42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -3340,9 +3388,9 @@
       <c r="I43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -3369,7 +3417,7 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.97"/>
@@ -3413,7 +3461,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D2" s="10" t="n">
@@ -3447,7 +3495,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D3" s="10" t="n">
@@ -3476,9 +3524,9 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -3487,9 +3535,9 @@
       <c r="I4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -3498,9 +3546,9 @@
       <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -3509,9 +3557,9 @@
       <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -3520,9 +3568,9 @@
       <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -3531,9 +3579,9 @@
       <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -3542,9 +3590,9 @@
       <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -3553,9 +3601,9 @@
       <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -3564,9 +3612,9 @@
       <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -3575,9 +3623,9 @@
       <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -3586,9 +3634,9 @@
       <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -3597,9 +3645,9 @@
       <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -3608,9 +3656,9 @@
       <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -3619,9 +3667,9 @@
       <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -3630,9 +3678,9 @@
       <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -3641,9 +3689,9 @@
       <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -3652,9 +3700,9 @@
       <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -3663,9 +3711,9 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -3674,9 +3722,9 @@
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -3685,9 +3733,9 @@
       <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -3696,9 +3744,9 @@
       <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -3707,9 +3755,9 @@
       <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -3718,9 +3766,9 @@
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -3729,9 +3777,9 @@
       <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -3740,9 +3788,9 @@
       <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -3751,9 +3799,9 @@
       <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -3762,9 +3810,9 @@
       <c r="I29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -3773,9 +3821,9 @@
       <c r="I30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -3784,9 +3832,9 @@
       <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -3795,9 +3843,9 @@
       <c r="I32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -3806,9 +3854,9 @@
       <c r="I33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -3817,9 +3865,9 @@
       <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -3828,9 +3876,9 @@
       <c r="I35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -3839,9 +3887,9 @@
       <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -3850,9 +3898,9 @@
       <c r="I37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -3861,9 +3909,9 @@
       <c r="I38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -3872,9 +3920,9 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -3883,9 +3931,9 @@
       <c r="I40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -3894,9 +3942,9 @@
       <c r="I41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -3905,9 +3953,9 @@
       <c r="I42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -3916,9 +3964,9 @@
       <c r="I43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -3945,14 +3993,14 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="19.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="22.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="28.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="18" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="19" width="15.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3990,7 +4038,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D2" s="10" t="n">
@@ -4024,7 +4072,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="20" t="n">
         <v>45702</v>
       </c>
       <c r="D3" s="10" t="n">
@@ -4053,9 +4101,9 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -4064,9 +4112,9 @@
       <c r="I4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
@@ -4075,9 +4123,9 @@
       <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -4086,9 +4134,9 @@
       <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -4097,9 +4145,9 @@
       <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -4108,9 +4156,9 @@
       <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -4119,9 +4167,9 @@
       <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -4130,9 +4178,9 @@
       <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -4141,9 +4189,9 @@
       <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -4152,9 +4200,9 @@
       <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -4163,9 +4211,9 @@
       <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -4174,9 +4222,9 @@
       <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -4185,9 +4233,9 @@
       <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -4196,9 +4244,9 @@
       <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -4207,9 +4255,9 @@
       <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -4218,9 +4266,9 @@
       <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -4229,9 +4277,9 @@
       <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -4240,9 +4288,9 @@
       <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -4251,9 +4299,9 @@
       <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -4262,9 +4310,9 @@
       <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -4273,9 +4321,9 @@
       <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -4284,9 +4332,9 @@
       <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -4295,9 +4343,9 @@
       <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -4306,9 +4354,9 @@
       <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -4317,9 +4365,9 @@
       <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -4328,9 +4376,9 @@
       <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -4339,9 +4387,9 @@
       <c r="I29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -4350,9 +4398,9 @@
       <c r="I30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -4361,9 +4409,9 @@
       <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -4372,9 +4420,9 @@
       <c r="I32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -4383,9 +4431,9 @@
       <c r="I33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -4394,9 +4442,9 @@
       <c r="I34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -4405,9 +4453,9 @@
       <c r="I35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -4416,9 +4464,9 @@
       <c r="I36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -4427,9 +4475,9 @@
       <c r="I37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -4438,9 +4486,9 @@
       <c r="I38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -4449,9 +4497,9 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -4460,9 +4508,9 @@
       <c r="I40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
       <c r="F41" s="10"/>
@@ -4471,9 +4519,9 @@
       <c r="I41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
@@ -4482,9 +4530,9 @@
       <c r="I42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -4493,9 +4541,9 @@
       <c r="I43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -4522,9 +4570,9 @@
   <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="21" width="26.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="18" width="27.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="18" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="19" width="27.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="19" width="15.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4544,10 +4592,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4559,7 +4607,7 @@
         <v>28</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4568,10 +4616,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4583,7 +4631,7 @@
         <v>31</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4592,7 +4640,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="15"/>
-      <c r="C6" s="20"/>
+      <c r="C6" s="21"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
@@ -4600,7 +4648,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="15"/>
-      <c r="C7" s="20"/>
+      <c r="C7" s="21"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
@@ -4608,7 +4656,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="15"/>
-      <c r="C8" s="20"/>
+      <c r="C8" s="21"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
@@ -4616,7 +4664,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="15"/>
-      <c r="C9" s="20"/>
+      <c r="C9" s="21"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
@@ -4624,7 +4672,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="15"/>
-      <c r="C10" s="20"/>
+      <c r="C10" s="21"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
@@ -4632,7 +4680,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="15"/>
-      <c r="C11" s="20"/>
+      <c r="C11" s="21"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
@@ -4640,7 +4688,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="15"/>
-      <c r="C12" s="20"/>
+      <c r="C12" s="21"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
@@ -4648,7 +4696,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="15"/>
-      <c r="C13" s="20"/>
+      <c r="C13" s="21"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
@@ -4656,7 +4704,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="15"/>
-      <c r="C14" s="20"/>
+      <c r="C14" s="21"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="n">
@@ -4664,7 +4712,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="15"/>
-      <c r="C15" s="20"/>
+      <c r="C15" s="21"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
@@ -4672,7 +4720,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="15"/>
-      <c r="C16" s="20"/>
+      <c r="C16" s="21"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="n">
@@ -4680,7 +4728,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="15"/>
-      <c r="C17" s="20"/>
+      <c r="C17" s="21"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
@@ -4688,7 +4736,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="15"/>
-      <c r="C18" s="20"/>
+      <c r="C18" s="21"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="n">
@@ -4696,7 +4744,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="15"/>
-      <c r="C19" s="20"/>
+      <c r="C19" s="21"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
@@ -4704,7 +4752,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="15"/>
-      <c r="C20" s="20"/>
+      <c r="C20" s="21"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="n">
@@ -4712,7 +4760,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="15"/>
-      <c r="C21" s="20"/>
+      <c r="C21" s="21"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="n">
@@ -4720,7 +4768,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="15"/>
-      <c r="C22" s="20"/>
+      <c r="C22" s="21"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="n">
@@ -4728,7 +4776,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="15"/>
-      <c r="C23" s="20"/>
+      <c r="C23" s="21"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="n">
@@ -4736,7 +4784,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="15"/>
-      <c r="C24" s="20"/>
+      <c r="C24" s="21"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="n">
@@ -4744,7 +4792,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="15"/>
-      <c r="C25" s="20"/>
+      <c r="C25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="n">
@@ -4752,7 +4800,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="15"/>
-      <c r="C26" s="20"/>
+      <c r="C26" s="21"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="n">
@@ -4760,7 +4808,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="15"/>
-      <c r="C27" s="20"/>
+      <c r="C27" s="21"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="n">
@@ -4768,87 +4816,87 @@
         <v>27</v>
       </c>
       <c r="B28" s="15"/>
-      <c r="C28" s="20"/>
+      <c r="C28" s="21"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
+      <c r="A29" s="18"/>
       <c r="B29" s="15"/>
-      <c r="C29" s="20"/>
+      <c r="C29" s="21"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
+      <c r="A30" s="18"/>
       <c r="B30" s="15"/>
-      <c r="C30" s="20"/>
+      <c r="C30" s="21"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="15"/>
-      <c r="C31" s="20"/>
+      <c r="C31" s="21"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="15"/>
-      <c r="C32" s="20"/>
+      <c r="C32" s="21"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="15"/>
-      <c r="C33" s="20"/>
+      <c r="C33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="15"/>
-      <c r="C34" s="20"/>
+      <c r="C34" s="21"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
+      <c r="A35" s="18"/>
       <c r="B35" s="15"/>
-      <c r="C35" s="20"/>
+      <c r="C35" s="21"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17"/>
+      <c r="A36" s="18"/>
       <c r="B36" s="15"/>
-      <c r="C36" s="20"/>
+      <c r="C36" s="21"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
+      <c r="A37" s="18"/>
       <c r="B37" s="15"/>
-      <c r="C37" s="20"/>
+      <c r="C37" s="21"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="15"/>
-      <c r="C38" s="20"/>
+      <c r="C38" s="21"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
+      <c r="A39" s="18"/>
       <c r="B39" s="15"/>
-      <c r="C39" s="20"/>
+      <c r="C39" s="21"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
+      <c r="A40" s="18"/>
       <c r="B40" s="15"/>
-      <c r="C40" s="20"/>
+      <c r="C40" s="21"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
+      <c r="A41" s="18"/>
       <c r="B41" s="15"/>
-      <c r="C41" s="20"/>
+      <c r="C41" s="21"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
+      <c r="A42" s="18"/>
       <c r="B42" s="15"/>
-      <c r="C42" s="20"/>
+      <c r="C42" s="21"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="20"/>
+      <c r="C43" s="21"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="20"/>
+      <c r="C44" s="21"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>